<commit_message>
feat(autorizaciones): registro de autorización excepcional, historial de registros y búsqueda del menú
- Módulo «Documentos de autorización» (RAUT): creación y modificación de vigencia según Figma; solo el creador
  autorizador (Rosa, permiso authorization.create) graba y autoriza directo a Aprobado, sin sustento ni aprobador.
- Registros con vigencia (desde / hasta); opción flujoDirecto en documents-records-page.
- Panel de historial de registros de saldos iniciales.
- Menú de procesos: estado «Sin resultados», ícono de búsqueda y botón para limpiar.
- Datos simulados versión 10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/menu-procesos.xlsx
+++ b/docs/menu-procesos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="55">
   <si>
     <t>id</t>
   </si>
@@ -107,37 +107,40 @@
     <t>Documentos de autorización</t>
   </si>
   <si>
+    <t>/procesos/autorizaciones</t>
+  </si>
+  <si>
+    <t>traspasos-cuentas-registros</t>
+  </si>
+  <si>
+    <t>Traspasos de cuentas de registros</t>
+  </si>
+  <si>
+    <t>doc-traslado-cta-registros</t>
+  </si>
+  <si>
+    <t>Documentos de traslado entre cuentas de registros</t>
+  </si>
+  <si>
+    <t>/procesos/registro-cuentas-bancarias</t>
+  </si>
+  <si>
+    <t>cons-traslado-cta-registros</t>
+  </si>
+  <si>
+    <t>Consultas y reportes de traslado entre cuentas de registros</t>
+  </si>
+  <si>
+    <t>/procesos/registro-cuentas-bancarias/consultas</t>
+  </si>
+  <si>
+    <t>clasificadores-catalogos</t>
+  </si>
+  <si>
+    <t>Clasificadores y catálogos</t>
+  </si>
+  <si>
     <t>proximamente</t>
-  </si>
-  <si>
-    <t>traspasos-cuentas-registros</t>
-  </si>
-  <si>
-    <t>Traspasos de cuentas de registros</t>
-  </si>
-  <si>
-    <t>doc-traslado-cta-registros</t>
-  </si>
-  <si>
-    <t>Documentos de traslado entre cuentas de registros</t>
-  </si>
-  <si>
-    <t>/procesos/registro-cuentas-bancarias</t>
-  </si>
-  <si>
-    <t>cons-traslado-cta-registros</t>
-  </si>
-  <si>
-    <t>Consultas y reportes de traslado entre cuentas de registros</t>
-  </si>
-  <si>
-    <t>/procesos/registro-cuentas-bancarias/consultas</t>
-  </si>
-  <si>
-    <t>clasificadores-catalogos</t>
-  </si>
-  <si>
-    <t>Clasificadores y catálogos</t>
   </si>
   <si>
     <t>consultas-reportes</t>
@@ -742,7 +745,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -753,13 +756,16 @@
         <v>22</v>
       </c>
       <c r="D8">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F8" t="s">
         <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -839,7 +845,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F12" t="s">
         <v>12</v>
@@ -847,10 +853,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D13">
         <v>10</v>
@@ -911,62 +917,62 @@
   <sheetData>
     <row r="1" ht="17.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(traspasos): ruta y módulo traspasos-cuentas-registros
- El módulo cuentas-bancarias pasa a modules/tesoreria/traspasos-cuentas-registros (mismo flujo).
- Ruta /procesos/traspasos-cuentas-registros (documentos, solicitud y consultas); las rutas
  /procesos/registro-cuentas-bancarias/… redirigen a las nuevas.
- Menú de procesos, migas, notificaciones, README y CLAUDE.md actualizados.
- Título de la pestaña: SIAF-RP · Sistema Integrado de Administración Financiera de los Recursos Públicos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/menu-procesos.xlsx
+++ b/docs/menu-procesos.xlsx
@@ -122,7 +122,7 @@
     <t>Documentos de traslado entre cuentas de registros</t>
   </si>
   <si>
-    <t>/procesos/registro-cuentas-bancarias</t>
+    <t>/procesos/traspasos-cuentas-registros</t>
   </si>
   <si>
     <t>cons-traslado-cta-registros</t>
@@ -131,7 +131,7 @@
     <t>Consultas y reportes de traslado entre cuentas de registros</t>
   </si>
   <si>
-    <t>/procesos/registro-cuentas-bancarias/consultas</t>
+    <t>/procesos/traspasos-cuentas-registros/consultas</t>
   </si>
   <si>
     <t>clasificadores-catalogos</t>

</xml_diff>